<commit_message>
Changed Solution Project Names & Refactored Folders
</commit_message>
<xml_diff>
--- a/examples/seating_plan/spreadsheets/example-classroom_seating_plan-org.xlsx
+++ b/examples/seating_plan/spreadsheets/example-classroom_seating_plan-org.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>Organised Seating Plan</t>
   </si>
@@ -117,12 +117,92 @@
   </si>
   <si>
     <t>Sophie Rayner, excellent</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>12</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts>
+	</numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -501,34 +581,34 @@
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -536,31 +616,31 @@
         <v>11</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>8</v>
+        <v>41</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>4</v>
+        <v>51</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>13</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -568,25 +648,25 @@
         <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>11</v>

</xml_diff>